<commit_message>
Sorted new capacity batching, tidied code, looking good
</commit_message>
<xml_diff>
--- a/input_files/batched_new_capacity.xlsx
+++ b/input_files/batched_new_capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/CODERS scripts/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{755BEA32-E367-4C39-88DE-53F098D0EA74}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9B6428F-E453-4035-8F8C-84D82ED988C4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Sets the capacity for batches of new installed capacity by technology. For updating assumptions by quantity of new capacity.</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>tech_generic</t>
-  </si>
-  <si>
-    <t>batches</t>
   </si>
 </sst>
 </file>
@@ -360,67 +357,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C2" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
         <v>5</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
       <c r="G3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K3">
-        <v>9</v>
-      </c>
-      <c r="L3">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="C4">
         <v>1000</v>
@@ -449,16 +442,13 @@
       <c r="K4">
         <v>1000</v>
       </c>
-      <c r="L4">
-        <v>1000</v>
-      </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>1000</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -473,6 +463,18 @@
         <v>1000</v>
       </c>
       <c r="G5">
+        <v>1000</v>
+      </c>
+      <c r="H5">
+        <v>1000</v>
+      </c>
+      <c r="I5">
+        <v>1000</v>
+      </c>
+      <c r="J5">
+        <v>1000</v>
+      </c>
+      <c r="K5">
         <v>1000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
major rewrites again. working all provinces now and reworking interties. much more configurable. option to use nrel atb data instead
</commit_message>
<xml_diff>
--- a/input_files/batched_new_capacity.xlsx
+++ b/input_files/batched_new_capacity.xlsx
@@ -8,12 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/electricity_sector/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C42019E-AAEA-4788-B54C-046B822CCBFB}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="11_F25DC773A252ABDACC104858199A58E65ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E05956E2-364D-43B4-86BC-F96F38566427}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11385" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ON" sheetId="1" r:id="rId1"/>
+    <sheet name="AB" sheetId="2" r:id="rId1"/>
+    <sheet name="BC" sheetId="3" r:id="rId2"/>
+    <sheet name="MB" sheetId="4" r:id="rId3"/>
+    <sheet name="NB" sheetId="5" r:id="rId4"/>
+    <sheet name="NLLAB" sheetId="6" r:id="rId5"/>
+    <sheet name="NS" sheetId="7" r:id="rId6"/>
+    <sheet name="ON" sheetId="1" r:id="rId7"/>
+    <sheet name="PEI" sheetId="8" r:id="rId8"/>
+    <sheet name="QC" sheetId="9" r:id="rId9"/>
+    <sheet name="SK" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,24 +34,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="4">
   <si>
-    <t>Sets the capacity for batches of new installed capacity by technology. For updating assumptions by quantity of new capacity.</t>
+    <t>tech_code</t>
   </si>
   <si>
-    <t>mw per batch</t>
+    <t>wind_onshore</t>
   </si>
   <si>
-    <t>WIND_ONSHORE</t>
+    <t>solar_pv</t>
   </si>
   <si>
-    <t>SOLAR_PV</t>
-  </si>
-  <si>
-    <t>tech_generic</t>
-  </si>
-  <si>
-    <t>HYDRO_RUN</t>
+    <t>hydro_run</t>
   </si>
 </sst>
 </file>
@@ -359,8 +362,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D5351A3-710B-4029-8385-12B1E066CEBB}">
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
@@ -370,135 +373,557 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52B4A62F-CD9F-4DED-AA85-29920C799F54}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D897E163-965B-4FC4-8069-4EB134279C86}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B2948BF-B8A7-4C04-B3E0-EF037C2091E9}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E66F99F-0D88-451D-B712-03FA8DEE3917}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AE6DF43-078B-49F4-AC35-9A024797E167}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BE2F9DE-BDA4-4551-96D5-2F99D2DB804E}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1000</v>
+      </c>
+      <c r="C2">
+        <v>1000</v>
+      </c>
+      <c r="D2">
+        <v>1000</v>
+      </c>
+      <c r="E2">
+        <v>1000</v>
+      </c>
+      <c r="F2">
+        <v>1000</v>
+      </c>
+      <c r="G2">
+        <v>1000</v>
+      </c>
+      <c r="H2">
+        <v>1000</v>
+      </c>
+      <c r="I2">
+        <v>1000</v>
+      </c>
+      <c r="J2">
+        <v>1000</v>
+      </c>
+      <c r="K2">
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2000</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>2000</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>2000</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>2000</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>2000</v>
       </c>
       <c r="G3">
-        <v>6</v>
+        <v>2000</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>2000</v>
       </c>
       <c r="I3">
-        <v>8</v>
+        <v>2000</v>
       </c>
       <c r="J3">
-        <v>9</v>
+        <v>2000</v>
       </c>
       <c r="K3">
-        <v>10</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="C4">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D4">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="E4">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F4">
-        <v>1000</v>
-      </c>
-      <c r="G4">
-        <v>1000</v>
-      </c>
-      <c r="H4">
-        <v>1000</v>
-      </c>
-      <c r="I4">
-        <v>1000</v>
-      </c>
-      <c r="J4">
-        <v>1000</v>
-      </c>
-      <c r="K4">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>2000</v>
-      </c>
-      <c r="C5">
-        <v>2000</v>
-      </c>
-      <c r="D5">
-        <v>2000</v>
-      </c>
-      <c r="E5">
-        <v>2000</v>
-      </c>
-      <c r="F5">
-        <v>2000</v>
-      </c>
-      <c r="G5">
-        <v>2000</v>
-      </c>
-      <c r="H5">
-        <v>2000</v>
-      </c>
-      <c r="I5">
-        <v>2000</v>
-      </c>
-      <c r="J5">
-        <v>2000</v>
-      </c>
-      <c r="K5">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+        <v>500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F31EEC0E-7F01-4C54-A6A6-3BDB9EBAC05F}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>500</v>
-      </c>
-      <c r="C6">
-        <v>500</v>
-      </c>
-      <c r="D6">
-        <v>500</v>
-      </c>
-      <c r="E6">
-        <v>500</v>
-      </c>
-      <c r="F6">
-        <v>500</v>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{013B8A34-8996-4337-B82D-E441BAE1C56B}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>